<commit_message>
Updated project trackingand adding the Tableau dashboard and visuals
</commit_message>
<xml_diff>
--- a/Capstone Project Docs/Project tracking .xlsx
+++ b/Capstone Project Docs/Project tracking .xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/48b30c63d0d95b74/Desktop/Capstone project/Capston Project Docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/48b30c63d0d95b74/Desktop/Capstone project/Capstone Project Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="95" documentId="8_{8C5D9351-945E-4D40-BC4C-AE6917795569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9632710-17E3-4952-916C-F5D189D0D69D}"/>
+  <xr:revisionPtr revIDLastSave="199" documentId="8_{8C5D9351-945E-4D40-BC4C-AE6917795569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB01751F-1AF6-44EC-AFDE-F688F1087389}"/>
   <bookViews>
-    <workbookView xWindow="1992" yWindow="2712" windowWidth="17280" windowHeight="9960" xr2:uid="{EB547DAF-3998-41E0-B73A-7028B050DDE6}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{EB547DAF-3998-41E0-B73A-7028B050DDE6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t xml:space="preserve">Milestones </t>
   </si>
@@ -460,421 +460,431 @@
         <rFont val="Aptos"/>
         <family val="2"/>
       </rPr>
+      <t>Build and train the model (Oct. 20- Oct. 20)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Track the model using W&amp;B (Oct. 20- Oct. 22)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Test, evaluate, and interpret the results of the model (Oct. 23- Oct. 23)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Align technical performance with business impact (Oct. 26- Oct. 26)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Evaluate the success of the model and analysis (Oct. 27- Oct. 27)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Analyze error and bias (Oct. 28- Oct. 28)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Make any needed corrections (Oct. 30- Nov. 2)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Summarize the findings (Nov. 3 -Nov.3)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Determine if additional iterations are needed (Nov. 3 -Nov.3)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Conduct a peer review/code edit (Nov. 4- Nov. 4)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Define deployment architecture (Nov. 5 -Nov. 5)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Draft technical documents (Nov. 5 – Nov. 6)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Create data dashboards (Nov. 6 -Nov. 9)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Create the final report (Nov. 9 -Nov. 10)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Share findings with the board (Nov.10 -Nov.10)</t>
+    </r>
+  </si>
+  <si>
+    <t>Phase 2: Data understanding (October 1-7)</t>
+  </si>
+  <si>
+    <t>Phase 3: Data Preparation (October 8-16)</t>
+  </si>
+  <si>
+    <t>Phase 4: Modeling (October 19-23)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Phase 5: Evaluation (October 26- November 4)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">              Phase 1: Business Understanding (September 28-30)</t>
+  </si>
+  <si>
+    <t>Phase 6: Deployment (November 5 -10)</t>
+  </si>
+  <si>
+    <t>9/24-9/25</t>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t>Hyperparameter tuning and cross-validation (Oct. 21- Oct. 22)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
       <t>Split the data sets (Oct. 19- Oct. 19)</t>
     </r>
   </si>
   <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Build and train the model (Oct. 20- Oct. 20)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Hyperparameter tuning and cross-validation (Oct. 21- Oct. 22)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Track the model using W&amp;B (Oct. 20- Oct. 22)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Test, evaluate, and interpret the results of the model (Oct. 23- Oct. 23)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Align technical performance with business impact (Oct. 26- Oct. 26)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Evaluate the success of the model and analysis (Oct. 27- Oct. 27)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Analyze error and bias (Oct. 28- Oct. 28)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Make any needed corrections (Oct. 30- Nov. 2)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Summarize the findings (Nov. 3 -Nov.3)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Determine if additional iterations are needed (Nov. 3 -Nov.3)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Conduct a peer review/code edit (Nov. 4- Nov. 4)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Define deployment architecture (Nov. 5 -Nov. 5)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Draft technical documents (Nov. 5 – Nov. 6)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Create data dashboards (Nov. 6 -Nov. 9)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Create the final report (Nov. 9 -Nov. 10)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>o</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Share findings with the board (Nov.10 -Nov.10)</t>
-    </r>
-  </si>
-  <si>
-    <t>Phase 2: Data understanding (October 1-7)</t>
-  </si>
-  <si>
-    <t>Phase 3: Data Preparation (October 8-16)</t>
-  </si>
-  <si>
-    <t>Phase 4: Modeling (October 19-23)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>Phase 5: Evaluation (October 26- November 4)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">              Phase 1: Business Understanding (September 28-30)</t>
-  </si>
-  <si>
-    <t>Phase 6: Deployment (November 5 -10)</t>
-  </si>
-  <si>
-    <t>9/24-9/25</t>
+    <t>Determine the optimal number of clusters</t>
+  </si>
+  <si>
+    <t>Interperate cluster characteristics</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -913,6 +923,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="7"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -940,7 +979,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -976,6 +1015,18 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="6"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="13"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1046,13 +1097,9 @@
 </FeaturePropertyBags>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FFC8D197-1473-4DC3-BF02-C03131E458AC}" name="Table1" displayName="Table1" ref="F1:H41" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="F1:H41" xr:uid="{FFC8D197-1473-4DC3-BF02-C03131E458AC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FFC8D197-1473-4DC3-BF02-C03131E458AC}" name="Table1" displayName="Table1" ref="F1:H43" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="F1:H43" xr:uid="{FFC8D197-1473-4DC3-BF02-C03131E458AC}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{615FB1FE-06B8-4F57-9D9E-A0FD0AA96CCA}" name="Milestones " dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{F6E9A4E9-99C9-4E9A-8A7D-2854C4CB6342}" name="Completed " dataDxfId="0"/>
@@ -1379,7 +1426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{287280A3-3277-4972-AFEF-C452B2E99B6A}">
-  <dimension ref="F1:H41"/>
+  <dimension ref="F1:H43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="86.5546875" style="1" customWidth="1"/>
@@ -1400,7 +1447,7 @@
     </row>
     <row r="2" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F2" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G2" s="6" t="b">
         <v>1</v>
@@ -1475,7 +1522,7 @@
     </row>
     <row r="9" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F9" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G9" s="6" t="b">
         <v>1</v>
@@ -1545,12 +1592,12 @@
         <v>1</v>
       </c>
       <c r="H15" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F16" s="8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G16" s="6" t="b">
         <v>0</v>
@@ -1562,7 +1609,7 @@
         <v>15</v>
       </c>
       <c r="G17" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="4">
         <v>46290</v>
@@ -1573,7 +1620,7 @@
         <v>16</v>
       </c>
       <c r="G18" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" s="4">
         <v>46290</v>
@@ -1584,7 +1631,10 @@
         <v>17</v>
       </c>
       <c r="G19" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H19" s="4">
+        <v>46294</v>
       </c>
     </row>
     <row r="20" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
@@ -1592,12 +1642,15 @@
         <v>18</v>
       </c>
       <c r="G20" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H20" s="4">
+        <v>46294</v>
       </c>
     </row>
     <row r="21" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F21" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G21" s="6" t="b">
         <v>0</v>
@@ -1609,93 +1662,118 @@
         <v>19</v>
       </c>
       <c r="G22" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H22" s="4">
+        <v>46294</v>
       </c>
     </row>
     <row r="23" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F23" s="2" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="G23" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" s="4">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="24" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="F24" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="G24" s="12" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="F24" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="3" t="b">
-        <v>0</v>
-      </c>
+      <c r="H24" s="13"/>
     </row>
     <row r="25" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F25" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G25" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H25" s="4">
+        <v>46294</v>
       </c>
     </row>
     <row r="26" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F26" s="2" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="G26" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H26" s="4">
+        <v>46295</v>
       </c>
     </row>
     <row r="27" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="F27" s="2" t="s">
-        <v>24</v>
+      <c r="F27" s="11" t="s">
+        <v>42</v>
       </c>
       <c r="G27" s="3" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="F28" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="G28" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H28" s="9"/>
+      <c r="F28" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G28" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H28" s="4">
+        <v>46294</v>
+      </c>
     </row>
     <row r="29" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F29" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G29" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H29" s="4">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="30" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="F30" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="G30" s="6" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="F30" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G30" s="3" t="b">
-        <v>0</v>
-      </c>
+      <c r="H30" s="9"/>
     </row>
     <row r="31" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F31" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G31" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H31" s="4">
+        <v>46295</v>
       </c>
     </row>
     <row r="32" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F32" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G32" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H32" s="4">
+        <v>46295</v>
       </c>
     </row>
     <row r="33" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F33" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G33" s="3" t="b">
         <v>0</v>
@@ -1703,48 +1781,51 @@
     </row>
     <row r="34" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F34" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G34" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H34" s="4">
+        <v>46295</v>
       </c>
     </row>
     <row r="35" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F35" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G35" s="3" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="36" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="F36" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="G36" s="6" t="b">
+      <c r="F36" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G36" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="H36" s="9"/>
     </row>
     <row r="37" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F37" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G37" s="3" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="38" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="F38" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G38" s="3" t="b">
+      <c r="F38" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="G38" s="6" t="b">
         <v>0</v>
       </c>
+      <c r="H38" s="9"/>
     </row>
     <row r="39" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F39" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G39" s="3" t="b">
         <v>0</v>
@@ -1752,17 +1833,36 @@
     </row>
     <row r="40" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F40" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G40" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H40" s="4">
+        <v>46296</v>
       </c>
     </row>
     <row r="41" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="F41" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="G41" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="F42" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G42" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="6:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="F43" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G43" s="3" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>